<commit_message>
Update inventory, FBA shipments, weekly sales snapshots and Fossil replenishment data
</commit_message>
<xml_diff>
--- a/data/input/Inventory_snapshot_tonor.xlsx
+++ b/data/input/Inventory_snapshot_tonor.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 14\Tonor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A54884E8-022F-4150-8BD3-C3D9F3C51D9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74CC5384-BEFC-49CC-A658-BD32D50925B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D49B0F4C-5F9E-467E-8AD9-9E638F42404F}"/>
   </bookViews>
@@ -174,9 +174,6 @@
     <t>B0CFKZ72N7</t>
   </si>
   <si>
-    <t>Ampm</t>
-  </si>
-  <si>
     <t>Warehouse</t>
   </si>
   <si>
@@ -496,6 +493,9 @@
   </si>
   <si>
     <t>YNT</t>
+  </si>
+  <si>
+    <t>AMPM</t>
   </si>
 </sst>
 </file>
@@ -1227,22 +1227,22 @@
     </row>
     <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>17</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="5">
@@ -1252,10 +1252,10 @@
         <v>7</v>
       </c>
       <c r="J2" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K2" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L2" s="5" t="s">
         <v>14</v>
@@ -1263,22 +1263,22 @@
     </row>
     <row r="3" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G3" s="5"/>
       <c r="H3" s="5">
@@ -1288,10 +1288,10 @@
         <v>1026</v>
       </c>
       <c r="J3" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="K3" s="13" t="s">
         <v>120</v>
-      </c>
-      <c r="K3" s="13" t="s">
-        <v>121</v>
       </c>
       <c r="L3" s="5" t="s">
         <v>14</v>
@@ -1299,22 +1299,22 @@
     </row>
     <row r="4" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>19</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G4" s="5"/>
       <c r="H4" s="5">
@@ -1324,10 +1324,10 @@
         <v>10</v>
       </c>
       <c r="J4" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K4" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L4" s="5" t="s">
         <v>14</v>
@@ -1335,22 +1335,22 @@
     </row>
     <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>42</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G5" s="5">
         <v>0</v>
@@ -1360,10 +1360,10 @@
       </c>
       <c r="I5" s="5"/>
       <c r="J5" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L5" s="5" t="s">
         <v>14</v>
@@ -1371,22 +1371,22 @@
     </row>
     <row r="6" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B6" s="8" t="s">
         <v>42</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G6" s="5"/>
       <c r="H6" s="5">
@@ -1396,10 +1396,10 @@
         <v>0</v>
       </c>
       <c r="J6" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K6" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L6" s="5" t="s">
         <v>14</v>
@@ -1407,22 +1407,22 @@
     </row>
     <row r="7" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>44</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G7" s="5">
         <v>0</v>
@@ -1432,10 +1432,10 @@
       </c>
       <c r="I7" s="5"/>
       <c r="J7" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L7" s="5" t="s">
         <v>14</v>
@@ -1443,22 +1443,22 @@
     </row>
     <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B8" s="8" t="s">
         <v>44</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G8" s="5"/>
       <c r="H8" s="5">
@@ -1468,10 +1468,10 @@
         <v>2</v>
       </c>
       <c r="J8" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K8" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K8" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L8" s="5" t="s">
         <v>14</v>
@@ -1479,22 +1479,22 @@
     </row>
     <row r="9" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>33</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G9" s="5"/>
       <c r="H9" s="5">
@@ -1515,22 +1515,22 @@
     </row>
     <row r="10" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>33</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G10" s="5"/>
       <c r="H10" s="5">
@@ -1540,10 +1540,10 @@
         <v>0</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L10" s="5" t="s">
         <v>14</v>
@@ -1551,22 +1551,22 @@
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>33</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G11" s="5"/>
       <c r="H11" s="5">
@@ -1576,10 +1576,10 @@
         <v>0</v>
       </c>
       <c r="J11" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K11" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K11" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L11" s="5" t="s">
         <v>14</v>
@@ -1587,22 +1587,22 @@
     </row>
     <row r="12" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>33</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G12" s="5"/>
       <c r="H12" s="5">
@@ -1612,10 +1612,10 @@
         <v>240</v>
       </c>
       <c r="J12" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="K12" s="13" t="s">
         <v>120</v>
-      </c>
-      <c r="K12" s="13" t="s">
-        <v>121</v>
       </c>
       <c r="L12" s="5" t="s">
         <v>14</v>
@@ -1623,22 +1623,22 @@
     </row>
     <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G13" s="5"/>
       <c r="H13" s="5">
@@ -1659,22 +1659,22 @@
     </row>
     <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>17</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G14" s="5"/>
       <c r="H14" s="5">
@@ -1695,22 +1695,22 @@
     </row>
     <row r="15" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>17</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G15" s="5"/>
       <c r="H15" s="5">
@@ -1720,10 +1720,10 @@
         <v>3</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L15" s="5" t="s">
         <v>14</v>
@@ -1731,22 +1731,22 @@
     </row>
     <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="B16" s="8" t="s">
-        <v>63</v>
-      </c>
       <c r="C16" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E16" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="F16" s="5" t="s">
         <v>137</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>138</v>
       </c>
       <c r="G16" s="5"/>
       <c r="H16" s="5">
@@ -1756,10 +1756,10 @@
         <v>0</v>
       </c>
       <c r="J16" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K16" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K16" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L16" s="5" t="s">
         <v>14</v>
@@ -1767,16 +1767,16 @@
     </row>
     <row r="17" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>65</v>
-      </c>
       <c r="C17" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E17" s="5" t="e">
         <v>#N/A</v>
@@ -1790,10 +1790,10 @@
         <v>0</v>
       </c>
       <c r="J17" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K17" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K17" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L17" s="5" t="s">
         <v>14</v>
@@ -1801,22 +1801,22 @@
     </row>
     <row r="18" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>19</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G18" s="5"/>
       <c r="H18" s="5">
@@ -1837,22 +1837,22 @@
     </row>
     <row r="19" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>19</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G19" s="5"/>
       <c r="H19" s="5">
@@ -1862,10 +1862,10 @@
         <v>2</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L19" s="5" t="s">
         <v>14</v>
@@ -1873,22 +1873,22 @@
     </row>
     <row r="20" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B20" s="8" t="s">
-        <v>48</v>
-      </c>
       <c r="C20" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D20" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="D20" s="8" t="s">
-        <v>84</v>
-      </c>
       <c r="E20" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="F20" s="5" t="s">
         <v>127</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>128</v>
       </c>
       <c r="G20" s="5"/>
       <c r="H20" s="5">
@@ -1898,10 +1898,10 @@
         <v>0</v>
       </c>
       <c r="J20" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K20" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K20" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L20" s="5" t="s">
         <v>14</v>
@@ -1909,22 +1909,22 @@
     </row>
     <row r="21" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>27</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G21" s="5"/>
       <c r="H21" s="5">
@@ -1945,22 +1945,22 @@
     </row>
     <row r="22" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>27</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G22" s="5"/>
       <c r="H22" s="5">
@@ -1970,10 +1970,10 @@
         <v>27</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L22" s="5" t="s">
         <v>14</v>
@@ -1981,22 +1981,22 @@
     </row>
     <row r="23" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B23" s="8" t="s">
         <v>27</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G23" s="5"/>
       <c r="H23" s="5">
@@ -2006,10 +2006,10 @@
         <v>5</v>
       </c>
       <c r="J23" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K23" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K23" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L23" s="5" t="s">
         <v>14</v>
@@ -2017,22 +2017,22 @@
     </row>
     <row r="24" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>27</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G24" s="5"/>
       <c r="H24" s="5">
@@ -2042,10 +2042,10 @@
         <v>204</v>
       </c>
       <c r="J24" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="K24" s="13" t="s">
         <v>120</v>
-      </c>
-      <c r="K24" s="13" t="s">
-        <v>121</v>
       </c>
       <c r="L24" s="5" t="s">
         <v>14</v>
@@ -2053,22 +2053,22 @@
     </row>
     <row r="25" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>31</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G25" s="5"/>
       <c r="H25" s="5">
@@ -2089,22 +2089,22 @@
     </row>
     <row r="26" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>31</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G26" s="5"/>
       <c r="H26" s="5">
@@ -2114,10 +2114,10 @@
         <v>2</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L26" s="5" t="s">
         <v>14</v>
@@ -2125,22 +2125,22 @@
     </row>
     <row r="27" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B27" s="8" t="s">
         <v>31</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G27" s="5"/>
       <c r="H27" s="5">
@@ -2150,10 +2150,10 @@
         <v>3</v>
       </c>
       <c r="J27" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K27" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K27" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L27" s="5" t="s">
         <v>14</v>
@@ -2161,22 +2161,22 @@
     </row>
     <row r="28" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>22</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G28" s="5"/>
       <c r="H28" s="5">
@@ -2197,22 +2197,22 @@
     </row>
     <row r="29" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>22</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G29" s="5"/>
       <c r="H29" s="5">
@@ -2222,10 +2222,10 @@
         <v>5</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L29" s="5" t="s">
         <v>14</v>
@@ -2233,22 +2233,22 @@
     </row>
     <row r="30" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B30" s="8" t="s">
         <v>22</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G30" s="5"/>
       <c r="H30" s="5">
@@ -2258,10 +2258,10 @@
         <v>11</v>
       </c>
       <c r="J30" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K30" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K30" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L30" s="5" t="s">
         <v>14</v>
@@ -2269,22 +2269,22 @@
     </row>
     <row r="31" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G31" s="5"/>
       <c r="H31" s="5">
@@ -2305,22 +2305,22 @@
     </row>
     <row r="32" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B32" s="8" t="s">
         <v>38</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G32" s="5"/>
       <c r="H32" s="5">
@@ -2330,10 +2330,10 @@
         <v>48</v>
       </c>
       <c r="J32" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K32" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K32" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L32" s="5" t="s">
         <v>14</v>
@@ -2341,22 +2341,22 @@
     </row>
     <row r="33" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>21</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G33" s="5"/>
       <c r="H33" s="5">
@@ -2377,22 +2377,22 @@
     </row>
     <row r="34" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>21</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G34" s="5">
         <v>0</v>
@@ -2402,10 +2402,10 @@
       </c>
       <c r="I34" s="5"/>
       <c r="J34" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L34" s="5" t="s">
         <v>14</v>
@@ -2413,22 +2413,22 @@
     </row>
     <row r="35" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B35" s="8" t="s">
         <v>21</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G35" s="5"/>
       <c r="H35" s="5">
@@ -2438,10 +2438,10 @@
         <v>5</v>
       </c>
       <c r="J35" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K35" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K35" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L35" s="5" t="s">
         <v>14</v>
@@ -2449,22 +2449,22 @@
     </row>
     <row r="36" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B36" s="8" t="s">
         <v>21</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G36" s="5"/>
       <c r="H36" s="5">
@@ -2474,10 +2474,10 @@
         <v>30</v>
       </c>
       <c r="J36" s="12" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K36" s="13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="L36" s="5" t="s">
         <v>14</v>
@@ -2485,22 +2485,22 @@
     </row>
     <row r="37" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>28</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G37" s="5"/>
       <c r="H37" s="5">
@@ -2521,22 +2521,22 @@
     </row>
     <row r="38" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>28</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G38" s="5">
         <v>0</v>
@@ -2546,10 +2546,10 @@
       </c>
       <c r="I38" s="5"/>
       <c r="J38" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L38" s="5" t="s">
         <v>14</v>
@@ -2557,22 +2557,22 @@
     </row>
     <row r="39" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B39" s="8" t="s">
         <v>28</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G39" s="5"/>
       <c r="H39" s="5">
@@ -2582,10 +2582,10 @@
         <v>0</v>
       </c>
       <c r="J39" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K39" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K39" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L39" s="5" t="s">
         <v>14</v>
@@ -2593,22 +2593,22 @@
     </row>
     <row r="40" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>20</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G40" s="5"/>
       <c r="H40" s="5">
@@ -2629,22 +2629,22 @@
     </row>
     <row r="41" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>20</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G41" s="5">
         <v>0</v>
@@ -2654,10 +2654,10 @@
       </c>
       <c r="I41" s="5"/>
       <c r="J41" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K41" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L41" s="5" t="s">
         <v>14</v>
@@ -2665,22 +2665,22 @@
     </row>
     <row r="42" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B42" s="8" t="s">
         <v>20</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G42" s="5"/>
       <c r="H42" s="5">
@@ -2690,10 +2690,10 @@
         <v>6</v>
       </c>
       <c r="J42" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K42" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K42" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L42" s="5" t="s">
         <v>14</v>
@@ -2701,22 +2701,22 @@
     </row>
     <row r="43" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B43" s="5" t="s">
         <v>24</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E43" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="F43" s="5" t="s">
         <v>127</v>
-      </c>
-      <c r="F43" s="5" t="s">
-        <v>128</v>
       </c>
       <c r="G43" s="5"/>
       <c r="H43" s="5">
@@ -2737,22 +2737,22 @@
     </row>
     <row r="44" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B44" s="5" t="s">
         <v>24</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E44" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="F44" s="5" t="s">
         <v>127</v>
-      </c>
-      <c r="F44" s="5" t="s">
-        <v>128</v>
       </c>
       <c r="G44" s="5"/>
       <c r="H44" s="5">
@@ -2762,10 +2762,10 @@
         <v>2</v>
       </c>
       <c r="J44" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K44" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L44" s="5" t="s">
         <v>14</v>
@@ -2773,22 +2773,22 @@
     </row>
     <row r="45" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B45" s="8" t="s">
         <v>24</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E45" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="F45" s="5" t="s">
         <v>127</v>
-      </c>
-      <c r="F45" s="5" t="s">
-        <v>128</v>
       </c>
       <c r="G45" s="5"/>
       <c r="H45" s="5">
@@ -2798,10 +2798,10 @@
         <v>0</v>
       </c>
       <c r="J45" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K45" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K45" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L45" s="5" t="s">
         <v>14</v>
@@ -2809,22 +2809,22 @@
     </row>
     <row r="46" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B46" s="8" t="s">
         <v>24</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E46" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="F46" s="5" t="s">
         <v>127</v>
-      </c>
-      <c r="F46" s="5" t="s">
-        <v>128</v>
       </c>
       <c r="G46" s="5"/>
       <c r="H46" s="5">
@@ -2834,10 +2834,10 @@
         <v>80</v>
       </c>
       <c r="J46" s="12" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K46" s="13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="L46" s="5" t="s">
         <v>14</v>
@@ -2845,22 +2845,22 @@
     </row>
     <row r="47" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G47" s="5"/>
       <c r="H47" s="5">
@@ -2881,22 +2881,22 @@
     </row>
     <row r="48" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B48" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G48" s="5"/>
       <c r="H48" s="5">
@@ -2917,22 +2917,22 @@
     </row>
     <row r="49" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B49" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G49" s="5"/>
       <c r="H49" s="5">
@@ -2942,10 +2942,10 @@
         <v>38</v>
       </c>
       <c r="J49" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K49" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L49" s="5" t="s">
         <v>14</v>
@@ -2953,22 +2953,22 @@
     </row>
     <row r="50" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B50" s="8" t="s">
         <v>16</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G50" s="5"/>
       <c r="H50" s="5">
@@ -2978,10 +2978,10 @@
         <v>279</v>
       </c>
       <c r="J50" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K50" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K50" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L50" s="5" t="s">
         <v>14</v>
@@ -2989,22 +2989,22 @@
     </row>
     <row r="51" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F51" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G51" s="5"/>
       <c r="H51" s="5">
@@ -3014,10 +3014,10 @@
         <v>9</v>
       </c>
       <c r="J51" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K51" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L51" s="5" t="s">
         <v>14</v>
@@ -3025,22 +3025,22 @@
     </row>
     <row r="52" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B52" s="8" t="s">
         <v>43</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F52" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G52" s="5"/>
       <c r="H52" s="5">
@@ -3050,10 +3050,10 @@
         <v>0</v>
       </c>
       <c r="J52" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K52" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K52" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L52" s="5" t="s">
         <v>14</v>
@@ -3061,22 +3061,22 @@
     </row>
     <row r="53" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>34</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G53" s="5"/>
       <c r="H53" s="5">
@@ -3097,22 +3097,22 @@
     </row>
     <row r="54" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B54" s="5" t="s">
         <v>34</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F54" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G54" s="5"/>
       <c r="H54" s="5">
@@ -3122,10 +3122,10 @@
         <v>4</v>
       </c>
       <c r="J54" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K54" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L54" s="5" t="s">
         <v>14</v>
@@ -3133,22 +3133,22 @@
     </row>
     <row r="55" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B55" s="8" t="s">
         <v>34</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F55" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G55" s="5"/>
       <c r="H55" s="5">
@@ -3158,10 +3158,10 @@
         <v>31</v>
       </c>
       <c r="J55" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K55" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K55" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L55" s="5" t="s">
         <v>14</v>
@@ -3169,22 +3169,22 @@
     </row>
     <row r="56" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B56" s="5" t="s">
         <v>35</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F56" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G56" s="5"/>
       <c r="H56" s="5">
@@ -3205,22 +3205,22 @@
     </row>
     <row r="57" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B57" s="5" t="s">
         <v>35</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F57" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G57" s="5"/>
       <c r="H57" s="5">
@@ -3230,10 +3230,10 @@
         <v>4</v>
       </c>
       <c r="J57" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K57" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L57" s="5" t="s">
         <v>14</v>
@@ -3241,22 +3241,22 @@
     </row>
     <row r="58" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B58" s="8" t="s">
         <v>35</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F58" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G58" s="5"/>
       <c r="H58" s="5">
@@ -3266,10 +3266,10 @@
         <v>10</v>
       </c>
       <c r="J58" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K58" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K58" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L58" s="5" t="s">
         <v>14</v>
@@ -3277,22 +3277,22 @@
     </row>
     <row r="59" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B59" s="5" t="s">
         <v>29</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F59" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G59" s="5"/>
       <c r="H59" s="5">
@@ -3313,22 +3313,22 @@
     </row>
     <row r="60" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B60" s="5" t="s">
         <v>29</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F60" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G60" s="5"/>
       <c r="H60" s="5">
@@ -3338,10 +3338,10 @@
         <v>6</v>
       </c>
       <c r="J60" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K60" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L60" s="5" t="s">
         <v>14</v>
@@ -3349,22 +3349,22 @@
     </row>
     <row r="61" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>29</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F61" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G61" s="5"/>
       <c r="H61" s="5">
@@ -3374,10 +3374,10 @@
         <v>20</v>
       </c>
       <c r="J61" s="12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K61" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L61" s="5" t="s">
         <v>14</v>
@@ -3385,22 +3385,22 @@
     </row>
     <row r="62" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B62" s="5" t="s">
         <v>29</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F62" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G62" s="5"/>
       <c r="H62" s="5">
@@ -3410,10 +3410,10 @@
         <v>3</v>
       </c>
       <c r="J62" s="12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K62" s="14" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L62" s="5" t="s">
         <v>14</v>
@@ -3421,22 +3421,22 @@
     </row>
     <row r="63" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B63" s="8" t="s">
         <v>29</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F63" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G63" s="5"/>
       <c r="H63" s="5">
@@ -3446,10 +3446,10 @@
         <v>5</v>
       </c>
       <c r="J63" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K63" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K63" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L63" s="5" t="s">
         <v>14</v>
@@ -3457,22 +3457,22 @@
     </row>
     <row r="64" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B64" s="5" t="s">
         <v>30</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F64" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G64" s="5"/>
       <c r="H64" s="5">
@@ -3493,22 +3493,22 @@
     </row>
     <row r="65" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B65" s="5" t="s">
         <v>30</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F65" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G65" s="5"/>
       <c r="H65" s="5">
@@ -3518,10 +3518,10 @@
         <v>7</v>
       </c>
       <c r="J65" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K65" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L65" s="5" t="s">
         <v>14</v>
@@ -3529,22 +3529,22 @@
     </row>
     <row r="66" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B66" s="8" t="s">
         <v>30</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F66" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G66" s="5"/>
       <c r="H66" s="5">
@@ -3554,10 +3554,10 @@
         <v>188</v>
       </c>
       <c r="J66" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K66" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K66" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L66" s="5" t="s">
         <v>14</v>
@@ -3565,22 +3565,22 @@
     </row>
     <row r="67" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>25</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E67" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="F67" s="5" t="s">
         <v>127</v>
-      </c>
-      <c r="F67" s="5" t="s">
-        <v>128</v>
       </c>
       <c r="G67" s="5"/>
       <c r="H67" s="5">
@@ -3601,22 +3601,22 @@
     </row>
     <row r="68" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>25</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E68" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="F68" s="5" t="s">
         <v>127</v>
-      </c>
-      <c r="F68" s="5" t="s">
-        <v>128</v>
       </c>
       <c r="G68" s="5"/>
       <c r="H68" s="5">
@@ -3626,10 +3626,10 @@
         <v>3</v>
       </c>
       <c r="J68" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K68" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L68" s="5" t="s">
         <v>14</v>
@@ -3637,22 +3637,22 @@
     </row>
     <row r="69" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B69" s="8" t="s">
         <v>25</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E69" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="F69" s="5" t="s">
         <v>127</v>
-      </c>
-      <c r="F69" s="5" t="s">
-        <v>128</v>
       </c>
       <c r="G69" s="5"/>
       <c r="H69" s="5">
@@ -3662,10 +3662,10 @@
         <v>13</v>
       </c>
       <c r="J69" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K69" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K69" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L69" s="5" t="s">
         <v>14</v>
@@ -3673,22 +3673,22 @@
     </row>
     <row r="70" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B70" s="5" t="s">
         <v>26</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F70" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G70" s="5"/>
       <c r="H70" s="5">
@@ -3709,22 +3709,22 @@
     </row>
     <row r="71" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>26</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F71" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G71" s="5"/>
       <c r="H71" s="5">
@@ -3734,10 +3734,10 @@
         <v>9</v>
       </c>
       <c r="J71" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K71" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L71" s="5" t="s">
         <v>14</v>
@@ -3745,22 +3745,22 @@
     </row>
     <row r="72" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B72" s="8" t="s">
         <v>26</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F72" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G72" s="5"/>
       <c r="H72" s="5">
@@ -3770,10 +3770,10 @@
         <v>52</v>
       </c>
       <c r="J72" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K72" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K72" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L72" s="5" t="s">
         <v>14</v>
@@ -3781,22 +3781,22 @@
     </row>
     <row r="73" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B73" s="5" t="s">
         <v>15</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F73" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G73" s="5"/>
       <c r="H73" s="5">
@@ -3817,22 +3817,22 @@
     </row>
     <row r="74" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B74" s="5" t="s">
         <v>15</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F74" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G74" s="5"/>
       <c r="H74" s="5">
@@ -3853,22 +3853,22 @@
     </row>
     <row r="75" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B75" s="5" t="s">
         <v>15</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F75" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G75" s="5"/>
       <c r="H75" s="5">
@@ -3878,10 +3878,10 @@
         <v>42</v>
       </c>
       <c r="J75" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K75" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L75" s="5" t="s">
         <v>14</v>
@@ -3889,22 +3889,22 @@
     </row>
     <row r="76" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B76" s="8" t="s">
         <v>15</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D76" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F76" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G76" s="5"/>
       <c r="H76" s="5">
@@ -3914,10 +3914,10 @@
         <v>359</v>
       </c>
       <c r="J76" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K76" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K76" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L76" s="5" t="s">
         <v>14</v>
@@ -3925,22 +3925,22 @@
     </row>
     <row r="77" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B77" s="5" t="s">
         <v>15</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E77" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F77" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G77" s="5"/>
       <c r="H77" s="5">
@@ -3950,10 +3950,10 @@
         <v>2</v>
       </c>
       <c r="J77" s="12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K77" s="14" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L77" s="5" t="s">
         <v>14</v>
@@ -3961,22 +3961,22 @@
     </row>
     <row r="78" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B78" s="3" t="s">
         <v>32</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E78" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F78" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G78" s="5"/>
       <c r="H78" s="5">
@@ -3986,10 +3986,10 @@
         <v>30</v>
       </c>
       <c r="J78" s="12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K78" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L78" s="5" t="s">
         <v>14</v>
@@ -3997,22 +3997,22 @@
     </row>
     <row r="79" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B79" s="5" t="s">
         <v>32</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E79" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F79" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G79" s="5"/>
       <c r="H79" s="5">
@@ -4033,22 +4033,22 @@
     </row>
     <row r="80" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B80" s="5" t="s">
         <v>32</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F80" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G80" s="5"/>
       <c r="H80" s="5">
@@ -4058,10 +4058,10 @@
         <v>14</v>
       </c>
       <c r="J80" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K80" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L80" s="5" t="s">
         <v>14</v>
@@ -4069,22 +4069,22 @@
     </row>
     <row r="81" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B81" s="5" t="s">
         <v>32</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F81" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G81" s="5"/>
       <c r="H81" s="5">
@@ -4094,10 +4094,10 @@
         <v>4</v>
       </c>
       <c r="J81" s="12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K81" s="14" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L81" s="5" t="s">
         <v>14</v>
@@ -4105,22 +4105,22 @@
     </row>
     <row r="82" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B82" s="8" t="s">
         <v>32</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F82" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G82" s="5"/>
       <c r="H82" s="5">
@@ -4130,10 +4130,10 @@
         <v>379</v>
       </c>
       <c r="J82" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K82" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K82" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L82" s="5" t="s">
         <v>14</v>
@@ -4141,22 +4141,22 @@
     </row>
     <row r="83" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B83" s="5" t="s">
         <v>41</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E83" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F83" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G83" s="5"/>
       <c r="H83" s="5">
@@ -4177,22 +4177,22 @@
     </row>
     <row r="84" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B84" s="5" t="s">
         <v>41</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E84" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F84" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G84" s="5"/>
       <c r="H84" s="5">
@@ -4202,10 +4202,10 @@
         <v>0</v>
       </c>
       <c r="J84" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K84" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L84" s="5" t="s">
         <v>14</v>
@@ -4213,22 +4213,22 @@
     </row>
     <row r="85" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B85" s="8" t="s">
         <v>41</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E85" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F85" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G85" s="5"/>
       <c r="H85" s="5">
@@ -4238,10 +4238,10 @@
         <v>1</v>
       </c>
       <c r="J85" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K85" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K85" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L85" s="5" t="s">
         <v>14</v>
@@ -4249,22 +4249,22 @@
     </row>
     <row r="86" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B86" s="6" t="s">
         <v>41</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F86" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G86" s="5"/>
       <c r="H86" s="5">
@@ -4274,10 +4274,10 @@
         <v>504</v>
       </c>
       <c r="J86" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="K86" s="13" t="s">
         <v>120</v>
-      </c>
-      <c r="K86" s="13" t="s">
-        <v>121</v>
       </c>
       <c r="L86" s="5" t="s">
         <v>14</v>
@@ -4285,22 +4285,22 @@
     </row>
     <row r="87" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B87" s="5" t="s">
         <v>40</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E87" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F87" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G87" s="5"/>
       <c r="H87" s="5">
@@ -4321,22 +4321,22 @@
     </row>
     <row r="88" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B88" s="5" t="s">
         <v>40</v>
       </c>
       <c r="C88" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E88" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F88" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G88" s="5"/>
       <c r="H88" s="5">
@@ -4346,10 +4346,10 @@
         <v>44</v>
       </c>
       <c r="J88" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K88" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L88" s="5" t="s">
         <v>14</v>
@@ -4357,22 +4357,22 @@
     </row>
     <row r="89" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B89" s="8" t="s">
         <v>40</v>
       </c>
       <c r="C89" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E89" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F89" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G89" s="5"/>
       <c r="H89" s="5">
@@ -4382,10 +4382,10 @@
         <v>100</v>
       </c>
       <c r="J89" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K89" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K89" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L89" s="5" t="s">
         <v>14</v>
@@ -4393,22 +4393,22 @@
     </row>
     <row r="90" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B90" s="8" t="s">
         <v>40</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E90" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F90" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G90" s="5"/>
       <c r="H90" s="5">
@@ -4418,10 +4418,10 @@
         <v>256</v>
       </c>
       <c r="J90" s="12" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K90" s="13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="L90" s="5" t="s">
         <v>14</v>
@@ -4429,22 +4429,22 @@
     </row>
     <row r="91" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B91" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E91" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F91" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G91" s="5"/>
       <c r="H91" s="5">
@@ -4465,22 +4465,22 @@
     </row>
     <row r="92" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B92" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C92" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D92" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E92" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F92" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G92" s="5"/>
       <c r="H92" s="5">
@@ -4501,22 +4501,22 @@
     </row>
     <row r="93" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B93" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D93" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E93" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F93" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G93" s="5"/>
       <c r="H93" s="5">
@@ -4526,10 +4526,10 @@
         <v>7</v>
       </c>
       <c r="J93" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K93" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L93" s="5" t="s">
         <v>14</v>
@@ -4537,22 +4537,22 @@
     </row>
     <row r="94" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B94" s="8" t="s">
         <v>18</v>
       </c>
       <c r="C94" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E94" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F94" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G94" s="5"/>
       <c r="H94" s="5">
@@ -4562,10 +4562,10 @@
         <v>11</v>
       </c>
       <c r="J94" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K94" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K94" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L94" s="5" t="s">
         <v>14</v>
@@ -4573,22 +4573,22 @@
     </row>
     <row r="95" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B95" s="5" t="s">
         <v>37</v>
       </c>
       <c r="C95" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D95" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E95" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F95" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G95" s="5"/>
       <c r="H95" s="5">
@@ -4609,22 +4609,22 @@
     </row>
     <row r="96" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B96" s="5" t="s">
         <v>37</v>
       </c>
       <c r="C96" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D96" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E96" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F96" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G96" s="5">
         <v>0</v>
@@ -4634,10 +4634,10 @@
       </c>
       <c r="I96" s="5"/>
       <c r="J96" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K96" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L96" s="5" t="s">
         <v>14</v>
@@ -4645,22 +4645,22 @@
     </row>
     <row r="97" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B97" s="8" t="s">
         <v>37</v>
       </c>
       <c r="C97" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E97" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F97" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G97" s="5"/>
       <c r="H97" s="5">
@@ -4670,10 +4670,10 @@
         <v>2</v>
       </c>
       <c r="J97" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K97" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K97" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L97" s="5" t="s">
         <v>14</v>
@@ -4681,22 +4681,22 @@
     </row>
     <row r="98" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B98" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C98" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D98" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E98" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F98" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G98" s="5"/>
       <c r="H98" s="5">
@@ -4717,22 +4717,22 @@
     </row>
     <row r="99" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B99" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C99" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D99" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E99" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F99" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G99" s="5"/>
       <c r="H99" s="5">
@@ -4742,10 +4742,10 @@
         <v>0</v>
       </c>
       <c r="J99" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K99" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L99" s="5" t="s">
         <v>14</v>
@@ -4753,22 +4753,22 @@
     </row>
     <row r="100" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B100" s="8" t="s">
         <v>23</v>
       </c>
       <c r="C100" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E100" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F100" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G100" s="5"/>
       <c r="H100" s="5">
@@ -4778,10 +4778,10 @@
         <v>4</v>
       </c>
       <c r="J100" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K100" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K100" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L100" s="5" t="s">
         <v>14</v>
@@ -4789,22 +4789,22 @@
     </row>
     <row r="101" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B101" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C101" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E101" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F101" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G101" s="5"/>
       <c r="H101" s="5">
@@ -4814,10 +4814,10 @@
         <v>150</v>
       </c>
       <c r="J101" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="K101" s="13" t="s">
         <v>120</v>
-      </c>
-      <c r="K101" s="13" t="s">
-        <v>121</v>
       </c>
       <c r="L101" s="5" t="s">
         <v>14</v>
@@ -4825,22 +4825,22 @@
     </row>
     <row r="102" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B102" s="5" t="s">
         <v>36</v>
       </c>
       <c r="C102" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E102" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F102" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G102" s="5"/>
       <c r="H102" s="5">
@@ -4861,22 +4861,22 @@
     </row>
     <row r="103" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B103" s="5" t="s">
         <v>36</v>
       </c>
       <c r="C103" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D103" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E103" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F103" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G103" s="5"/>
       <c r="H103" s="5">
@@ -4886,10 +4886,10 @@
         <v>6</v>
       </c>
       <c r="J103" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K103" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L103" s="5" t="s">
         <v>14</v>
@@ -4897,22 +4897,22 @@
     </row>
     <row r="104" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B104" s="8" t="s">
         <v>36</v>
       </c>
       <c r="C104" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E104" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F104" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G104" s="5"/>
       <c r="H104" s="5">
@@ -4922,10 +4922,10 @@
         <v>20</v>
       </c>
       <c r="J104" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K104" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K104" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L104" s="5" t="s">
         <v>14</v>
@@ -4933,22 +4933,22 @@
     </row>
     <row r="105" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B105" s="5" t="s">
         <v>39</v>
       </c>
       <c r="C105" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D105" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E105" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F105" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G105" s="5"/>
       <c r="H105" s="5">
@@ -4969,22 +4969,22 @@
     </row>
     <row r="106" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B106" s="8" t="s">
         <v>39</v>
       </c>
       <c r="C106" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E106" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F106" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G106" s="5"/>
       <c r="H106" s="5">
@@ -4994,10 +4994,10 @@
         <v>8</v>
       </c>
       <c r="J106" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="K106" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="K106" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="L106" s="5" t="s">
         <v>14</v>

</xml_diff>

<commit_message>
Update Audio Array and Tonor inventory snapshots
</commit_message>
<xml_diff>
--- a/data/input/Inventory_snapshot_tonor.xlsx
+++ b/data/input/Inventory_snapshot_tonor.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 19\Tonor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{072C4DDC-9E02-4CD7-8FFC-2B36F4ADA122}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7D5BB9C-5F28-4349-B1C3-21BEF33A3276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D49B0F4C-5F9E-467E-8AD9-9E638F42404F}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$100</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1695,7 +1695,7 @@
         <v>91</v>
       </c>
       <c r="I33">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="J33" s="1" t="s">
         <v>101</v>
@@ -1715,7 +1715,7 @@
         <v>99</v>
       </c>
       <c r="I34">
-        <v>74</v>
+        <v>120</v>
       </c>
       <c r="J34" s="1" t="s">
         <v>101</v>
@@ -1735,7 +1735,7 @@
         <v>72</v>
       </c>
       <c r="I35">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="J35" s="1" t="s">
         <v>101</v>
@@ -1755,7 +1755,7 @@
         <v>83</v>
       </c>
       <c r="I36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J36" s="1" t="s">
         <v>101</v>
@@ -1775,7 +1775,7 @@
         <v>75</v>
       </c>
       <c r="I37">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J37" s="1" t="s">
         <v>101</v>
@@ -1795,7 +1795,7 @@
         <v>76</v>
       </c>
       <c r="I38">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J38" s="1" t="s">
         <v>101</v>
@@ -1855,7 +1855,7 @@
         <v>80</v>
       </c>
       <c r="I41">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J41" s="1" t="s">
         <v>101</v>
@@ -1874,7 +1874,9 @@
       <c r="D42" t="s">
         <v>118</v>
       </c>
-      <c r="I42"/>
+      <c r="I42">
+        <v>0</v>
+      </c>
       <c r="J42" s="1" t="s">
         <v>101</v>
       </c>
@@ -1892,7 +1894,9 @@
       <c r="D43" t="s">
         <v>74</v>
       </c>
-      <c r="I43"/>
+      <c r="I43">
+        <v>1</v>
+      </c>
       <c r="J43" s="1" t="s">
         <v>101</v>
       </c>
@@ -1910,7 +1914,9 @@
       <c r="D44" t="s">
         <v>73</v>
       </c>
-      <c r="I44"/>
+      <c r="I44">
+        <v>0</v>
+      </c>
       <c r="J44" s="1" t="s">
         <v>101</v>
       </c>
@@ -1929,7 +1935,7 @@
         <v>93</v>
       </c>
       <c r="I45">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="J45" s="1" t="s">
         <v>101</v>
@@ -1989,7 +1995,7 @@
         <v>71</v>
       </c>
       <c r="I48">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J48" s="1" t="s">
         <v>101</v>
@@ -2028,7 +2034,9 @@
       <c r="D50" t="s">
         <v>78</v>
       </c>
-      <c r="I50"/>
+      <c r="I50">
+        <v>0</v>
+      </c>
       <c r="J50" s="1" t="s">
         <v>101</v>
       </c>
@@ -2067,7 +2075,7 @@
         <v>94</v>
       </c>
       <c r="I52">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J52" s="1" t="s">
         <v>101</v>
@@ -2087,7 +2095,7 @@
         <v>92</v>
       </c>
       <c r="I53">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="J53" s="1" t="s">
         <v>101</v>
@@ -2107,7 +2115,7 @@
         <v>77</v>
       </c>
       <c r="I54">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="J54" s="1" t="s">
         <v>101</v>
@@ -2126,7 +2134,9 @@
       <c r="D55" t="s">
         <v>90</v>
       </c>
-      <c r="I55"/>
+      <c r="I55">
+        <v>0</v>
+      </c>
       <c r="J55" s="1" t="s">
         <v>101</v>
       </c>
@@ -2165,7 +2175,7 @@
         <v>97</v>
       </c>
       <c r="I57">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J57" s="1" t="s">
         <v>101</v>
@@ -3035,7 +3045,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L97" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}"/>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="A59">
     <cfRule type="duplicateValues" dxfId="10" priority="11"/>

</xml_diff>

<commit_message>
SP-API refresh 2026-08-04 — FBA inv + ledger + inbound + returns + vendor SOH
- Inventory (5): Nex 330 / Viomi 1166 / AA 292 / WM 147 / Fossil 21672 SKUs
- Ledger (5): all latest 2026-08-02 (~2d lag)
- Inbound --active-only (5): Nex 43 / Viomi 21 / AA 5 / WM 9 / Fossil 24 shipments
- Returns 90d (5): Nex 1773 / Viomi 739 / AA 445 / WM 198 / Fossil 1387
- Vendor SOH (AA/Tonor): 142 + 28 rows @ 2026-08-01
- Snapshot Model enrichment: WM 33 -> 41 populated

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/Inventory_snapshot_tonor.xlsx
+++ b/data/input/Inventory_snapshot_tonor.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\Nitesh Gdrive\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 30\Tonor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\Nitesh Gdrive\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 31\Tonor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87C970EE-D438-4D6A-8933-D7F4E2CE446D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87F00260-A3CE-48E1-84FC-6A2F924A0C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D49B0F4C-5F9E-467E-8AD9-9E638F42404F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FFC2A7B7-9814-40EF-9366-0F59D71BB19E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -78,139 +78,130 @@
     <t>FBA77101</t>
   </si>
   <si>
+    <t>B07WLWN2ZT</t>
+  </si>
+  <si>
+    <t>FBA79260</t>
+  </si>
+  <si>
+    <t>B07GVGMW59</t>
+  </si>
+  <si>
+    <t>FBA77105</t>
+  </si>
+  <si>
+    <t>B089FVQD3Z</t>
+  </si>
+  <si>
     <t>FBA77111</t>
   </si>
   <si>
+    <t>B08CVP2HXP</t>
+  </si>
+  <si>
+    <t>FBA77114</t>
+  </si>
+  <si>
+    <t>B07TSN2H9D</t>
+  </si>
+  <si>
+    <t>FBA77115</t>
+  </si>
+  <si>
+    <t>B08V1JS3NY</t>
+  </si>
+  <si>
+    <t>FBA77116</t>
+  </si>
+  <si>
+    <t>B0BBL47VR5</t>
+  </si>
+  <si>
+    <t>FBA77117</t>
+  </si>
+  <si>
+    <t>B078WNW4YW</t>
+  </si>
+  <si>
     <t>FBA77113</t>
   </si>
   <si>
+    <t>B01ISNU3X4</t>
+  </si>
+  <si>
+    <t>FBA77103</t>
+  </si>
+  <si>
+    <t>B09Z5Q194D</t>
+  </si>
+  <si>
     <t>FBA79111</t>
   </si>
   <si>
-    <t>FBA77103</t>
-  </si>
-  <si>
-    <t>FBA77105</t>
-  </si>
-  <si>
-    <t>FBA77115</t>
-  </si>
-  <si>
-    <t>FBA77116</t>
-  </si>
-  <si>
-    <t>FBA77117</t>
+    <t>B0BRKFP94K</t>
   </si>
   <si>
     <t>FBA79113</t>
   </si>
   <si>
+    <t>B0BTCXQQ6M</t>
+  </si>
+  <si>
     <t>FBA79114</t>
   </si>
   <si>
+    <t>B0CCV74CL7</t>
+  </si>
+  <si>
     <t>FBA79116</t>
   </si>
   <si>
-    <t>FBA79260</t>
+    <t>B0BYHHSLPC</t>
+  </si>
+  <si>
+    <t>FBA79576</t>
+  </si>
+  <si>
+    <t>B0BRCR2QQ7</t>
+  </si>
+  <si>
+    <t>FBA79577</t>
+  </si>
+  <si>
+    <t>B0CSCT63BL</t>
+  </si>
+  <si>
+    <t>FBA79586</t>
+  </si>
+  <si>
+    <t>B0CH9JR3HL</t>
   </si>
   <si>
     <t>FBA79574</t>
   </si>
   <si>
-    <t>FBA79576</t>
-  </si>
-  <si>
-    <t>FBA79577</t>
+    <t>B0B4WTHLX5</t>
   </si>
   <si>
     <t>FBA79585</t>
   </si>
   <si>
-    <t>FBA79586</t>
+    <t>B0CFKHCQ8W</t>
+  </si>
+  <si>
+    <t>FBA79697</t>
+  </si>
+  <si>
+    <t>B0CQX4K9P5</t>
   </si>
   <si>
     <t>FBA79696</t>
   </si>
   <si>
-    <t>FBA79697</t>
-  </si>
-  <si>
-    <t>B07WLWN2ZT</t>
-  </si>
-  <si>
-    <t>B08CVP2HXP</t>
-  </si>
-  <si>
-    <t>B01ISNU3X4</t>
-  </si>
-  <si>
-    <t>B0BRKFP94K</t>
-  </si>
-  <si>
-    <t>B09Z5Q194D</t>
-  </si>
-  <si>
-    <t>B089FVQD3Z</t>
-  </si>
-  <si>
-    <t>B08V1JS3NY</t>
-  </si>
-  <si>
-    <t>B0BBL47VR5</t>
-  </si>
-  <si>
-    <t>B078WNW4YW</t>
-  </si>
-  <si>
-    <t>B0BTCXQQ6M</t>
-  </si>
-  <si>
-    <t>B0CCV74CL7</t>
-  </si>
-  <si>
-    <t>B0BYHHSLPC</t>
-  </si>
-  <si>
-    <t>B07GVGMW59</t>
-  </si>
-  <si>
-    <t>B0B4WTHLX5</t>
-  </si>
-  <si>
-    <t>B0BRCR2QQ7</t>
-  </si>
-  <si>
-    <t>B0CSCT63BL</t>
-  </si>
-  <si>
-    <t>B0CFKHCQ8W</t>
-  </si>
-  <si>
-    <t>B0CH9JR3HL</t>
-  </si>
-  <si>
     <t>B0CQX3VB1R</t>
   </si>
   <si>
-    <t>B0CQX4K9P5</t>
-  </si>
-  <si>
     <t>Tonor</t>
-  </si>
-  <si>
-    <t>FBA77114</t>
-  </si>
-  <si>
-    <t>B07TSN2H9D</t>
-  </si>
-  <si>
-    <t>Open Order</t>
-  </si>
-  <si>
-    <t>AMPM</t>
-  </si>
-  <si>
-    <t>B2B - AMPM</t>
   </si>
   <si>
     <t>TC-777</t>
@@ -276,6 +267,15 @@
   </si>
   <si>
     <t>TD310+</t>
+  </si>
+  <si>
+    <t>AMPM</t>
+  </si>
+  <si>
+    <t>B2B - AMPM</t>
+  </si>
+  <si>
+    <t>Open Order</t>
   </si>
 </sst>
 </file>
@@ -283,21 +283,14 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="164" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -308,19 +301,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="8"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Bookman Old Style"/>
@@ -328,13 +308,27 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF111827"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF111827"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -385,66 +379,140 @@
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
-    <cellStyle name="Comma" xfId="3" builtinId="3"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2" xr:uid="{697FC575-8A7C-4715-A8F0-2950C62D8576}"/>
-    <cellStyle name="Normal 6" xfId="1" xr:uid="{E5F241CE-C0FC-4730-81C9-F1901EB82A3C}"/>
+    <cellStyle name="Normal 2" xfId="3" xr:uid="{F37F9E33-BAB9-493A-9CBA-C25E5FEA33D0}"/>
+    <cellStyle name="Normal 6" xfId="2" xr:uid="{C0B7BEB6-A9CE-4FBD-8F7F-EC4AAD93DADA}"/>
   </cellStyles>
-  <dxfs count="11">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
+  <dxfs count="18">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -567,39 +635,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -651,7 +719,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -762,6 +830,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -770,13 +845,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -841,91 +909,56 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E1E6F6A-7C3C-4952-AC4D-06F30C852840}">
   <dimension ref="A1:L25"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="42.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.88671875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="23.33203125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="28.44140625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.44140625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="8.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12" style="1" customWidth="1"/>
-    <col min="11" max="11" width="16.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="8.88671875" style="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -934,508 +967,499 @@
         <v>12</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>58</v>
+        <v>13</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>55</v>
       </c>
       <c r="I2" s="3">
-        <v>290</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>56</v>
+        <v>286</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>59</v>
+        <v>15</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>56</v>
       </c>
       <c r="I3" s="3">
-        <v>60</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>56</v>
+        <v>14</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>60</v>
+      <c r="C4" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>57</v>
       </c>
       <c r="I4" s="3">
-        <v>6</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>56</v>
+        <v>5</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>61</v>
+        <v>19</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>58</v>
       </c>
       <c r="I5" s="3">
-        <v>69</v>
-      </c>
-      <c r="J5" s="1" t="s">
         <v>56</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>63</v>
+        <v>23</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>60</v>
       </c>
       <c r="I6" s="3">
         <v>6</v>
       </c>
-      <c r="J6" s="1" t="s">
-        <v>56</v>
+      <c r="J6" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>64</v>
+        <v>25</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>61</v>
       </c>
       <c r="I7" s="3">
         <v>50</v>
       </c>
-      <c r="J7" s="1" t="s">
-        <v>56</v>
+      <c r="J7" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>65</v>
+        <v>27</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>62</v>
       </c>
       <c r="I8" s="3">
-        <v>118</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>56</v>
+        <v>115</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>66</v>
+        <v>29</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>63</v>
       </c>
       <c r="I9" s="3">
-        <v>518</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>56</v>
+        <v>496</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>67</v>
+        <v>31</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>64</v>
       </c>
       <c r="I10" s="3">
         <v>10</v>
       </c>
-      <c r="J10" s="1" t="s">
-        <v>56</v>
+      <c r="J10" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>68</v>
+        <v>33</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>65</v>
       </c>
       <c r="I11" s="3">
-        <v>7</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>56</v>
+        <v>6</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>69</v>
+        <v>35</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>66</v>
       </c>
       <c r="I12" s="3">
         <v>3</v>
       </c>
-      <c r="J12" s="1" t="s">
-        <v>56</v>
+      <c r="J12" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>70</v>
+        <v>37</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>67</v>
       </c>
       <c r="I13" s="3">
-        <v>80</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>56</v>
+        <v>76</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D14" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="I14" s="3">
         <v>71</v>
       </c>
-      <c r="I14" s="3">
-        <v>72</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>56</v>
+      <c r="J14" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>72</v>
+        <v>41</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>69</v>
       </c>
       <c r="I15" s="3">
         <v>8</v>
       </c>
-      <c r="J15" s="1" t="s">
-        <v>56</v>
+      <c r="J15" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>73</v>
+        <v>43</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>70</v>
       </c>
       <c r="I16" s="3">
-        <v>9</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>56</v>
+        <v>4</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>74</v>
+        <v>45</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>71</v>
       </c>
       <c r="I17" s="3">
         <v>5</v>
       </c>
-      <c r="J17" s="1" t="s">
-        <v>56</v>
+      <c r="J17" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D18" s="8" t="s">
-        <v>75</v>
+        <v>47</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>72</v>
       </c>
       <c r="I18" s="3">
         <v>26</v>
       </c>
-      <c r="J18" s="1" t="s">
-        <v>56</v>
+      <c r="J18" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>76</v>
+        <v>49</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>73</v>
       </c>
       <c r="I19" s="3">
         <v>7</v>
       </c>
-      <c r="J19" s="1" t="s">
-        <v>56</v>
+      <c r="J19" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C20" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>77</v>
+      <c r="C20" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>74</v>
       </c>
       <c r="I20" s="3">
         <v>287</v>
       </c>
-      <c r="J20" s="1" t="s">
-        <v>56</v>
+      <c r="J20" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D21" s="8" t="s">
-        <v>78</v>
+        <v>53</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>75</v>
       </c>
       <c r="I21" s="3">
-        <v>260</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>56</v>
+        <v>257</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="I22" s="9">
+      <c r="A22" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="I22" s="8">
         <v>2</v>
       </c>
-      <c r="J22" s="1" t="s">
-        <v>57</v>
+      <c r="J22" s="2" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C23" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="D23" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="I23" s="9">
+      <c r="A23" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="I23" s="8">
         <v>4</v>
       </c>
-      <c r="J23" s="1" t="s">
-        <v>57</v>
+      <c r="J23" s="2" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="12" t="s">
+      <c r="A24" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B24" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C24" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="I24" s="9">
+      <c r="B24" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="I24" s="8">
         <v>2</v>
       </c>
-      <c r="J24" s="1" t="s">
-        <v>57</v>
+      <c r="J24" s="2" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>53</v>
+        <v>20</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D25" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="I25" s="7">
+        <v>21</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="I25" s="12">
         <v>80</v>
       </c>
-      <c r="J25" s="6" t="s">
-        <v>55</v>
+      <c r="J25" s="11" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L25" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}"/>
-  <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="A12:A13">
-    <cfRule type="duplicateValues" dxfId="10" priority="2603"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="2604"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="duplicateValues" dxfId="8" priority="2365"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="140"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:H1">
-    <cfRule type="duplicateValues" dxfId="7" priority="2576"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="2577" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="141"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="142" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1">
-    <cfRule type="duplicateValues" dxfId="5" priority="2363"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="2364" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="138"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="139" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:L1">
-    <cfRule type="duplicateValues" dxfId="3" priority="2361"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="2362" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="136"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="137" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A25">
-    <cfRule type="duplicateValues" dxfId="1" priority="2639"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A21">
-    <cfRule type="duplicateValues" dxfId="0" priority="2642"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="144"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly SP-API refresh 2026-08-11 — sales W32 + 20-pull sweep + CB SOH
FBA Sales W32 (Aug 2-8): Nex 1014 / AA 327 / Viomi 278 / Fossil 234 / WM 65 rows
FBA Inv (5): Nex 332 / Viomi 1166 / AA 292 / WM 147 / Fossil 21714 SKUs
Ledger (5): latest 2026-08-09 across all 5 accounts (~2d SP-API lag)
Inbound --active-only (5): Nex 35 / Fossil 25 / Viomi 25 / WM 17 / AA 5 shipments
Returns 90d (5): Nex 1763 / Fossil 1342 / Viomi 742 / AA 463 / WM 211 rows
CB SOH (AA + Tonor): 142 + 28 rows @ 2026-08-08

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/Inventory_snapshot_tonor.xlsx
+++ b/data/input/Inventory_snapshot_tonor.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\Nitesh Gdrive\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 31\Tonor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Drive D\Week 32\Week 31 &amp; 32\Inventory\Tonor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87F00260-A3CE-48E1-84FC-6A2F924A0C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E66A4811-BDA6-4397-84CF-036A61080B11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FFC2A7B7-9814-40EF-9366-0F59D71BB19E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D49B0F4C-5F9E-467E-8AD9-9E638F42404F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -78,9 +78,48 @@
     <t>FBA77101</t>
   </si>
   <si>
+    <t>FBA79113</t>
+  </si>
+  <si>
+    <t>FBA79116</t>
+  </si>
+  <si>
     <t>B07WLWN2ZT</t>
   </si>
   <si>
+    <t>B0BTCXQQ6M</t>
+  </si>
+  <si>
+    <t>B0BYHHSLPC</t>
+  </si>
+  <si>
+    <t>Tonor</t>
+  </si>
+  <si>
+    <t>B2B - AMPM</t>
+  </si>
+  <si>
+    <t>TC-777</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC310	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-777 PRO	</t>
+  </si>
+  <si>
+    <t>FBA77114</t>
+  </si>
+  <si>
+    <t>B07TSN2H9D</t>
+  </si>
+  <si>
+    <t>TC-2030</t>
+  </si>
+  <si>
+    <t>Open Order</t>
+  </si>
+  <si>
     <t>FBA79260</t>
   </si>
   <si>
@@ -99,12 +138,6 @@
     <t>B08CVP2HXP</t>
   </si>
   <si>
-    <t>FBA77114</t>
-  </si>
-  <si>
-    <t>B07TSN2H9D</t>
-  </si>
-  <si>
     <t>FBA77115</t>
   </si>
   <si>
@@ -141,24 +174,12 @@
     <t>B0BRKFP94K</t>
   </si>
   <si>
-    <t>FBA79113</t>
-  </si>
-  <si>
-    <t>B0BTCXQQ6M</t>
-  </si>
-  <si>
     <t>FBA79114</t>
   </si>
   <si>
     <t>B0CCV74CL7</t>
   </si>
   <si>
-    <t>FBA79116</t>
-  </si>
-  <si>
-    <t>B0BYHHSLPC</t>
-  </si>
-  <si>
     <t>FBA79576</t>
   </si>
   <si>
@@ -201,12 +222,6 @@
     <t>B0CQX3VB1R</t>
   </si>
   <si>
-    <t>Tonor</t>
-  </si>
-  <si>
-    <t>TC-777</t>
-  </si>
-  <si>
     <t>G11</t>
   </si>
   <si>
@@ -214,9 +229,6 @@
   </si>
   <si>
     <t>TC30</t>
-  </si>
-  <si>
-    <t>TC-2030</t>
   </si>
   <si>
     <t>TC40</t>
@@ -239,15 +251,9 @@
     <t xml:space="preserve">TD510	</t>
   </si>
   <si>
-    <t xml:space="preserve">TC310	</t>
-  </si>
-  <si>
     <t>TC310+</t>
   </si>
   <si>
-    <t xml:space="preserve">TC-777 PRO	</t>
-  </si>
-  <si>
     <t>TC30S+</t>
   </si>
   <si>
@@ -270,12 +276,6 @@
   </si>
   <si>
     <t>AMPM</t>
-  </si>
-  <si>
-    <t>B2B - AMPM</t>
-  </si>
-  <si>
-    <t>Open Order</t>
   </si>
 </sst>
 </file>
@@ -283,14 +283,21 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -301,6 +308,19 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Bookman Old Style"/>
@@ -308,27 +328,13 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color rgb="FF111827"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF111827"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -379,54 +385,54 @@
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Comma" xfId="3" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="3" xr:uid="{F37F9E33-BAB9-493A-9CBA-C25E5FEA33D0}"/>
-    <cellStyle name="Normal 6" xfId="2" xr:uid="{C0B7BEB6-A9CE-4FBD-8F7F-EC4AAD93DADA}"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{697FC575-8A7C-4715-A8F0-2950C62D8576}"/>
+    <cellStyle name="Normal 6" xfId="1" xr:uid="{E5F241CE-C0FC-4730-81C9-F1901EB82A3C}"/>
   </cellStyles>
-  <dxfs count="18">
+  <dxfs count="11">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -439,80 +445,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -635,39 +567,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -719,7 +651,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -830,13 +762,6 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -845,6 +770,13 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -909,557 +841,600 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E1E6F6A-7C3C-4952-AC4D-06F30C852840}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}">
   <dimension ref="A1:L25"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="42.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="23.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="28.44140625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="16.44140625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="8.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12" style="1" customWidth="1"/>
+    <col min="11" max="11" width="16.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="8.88671875" style="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="5">
+        <v>2</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="5">
+        <v>4</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="I2" s="3">
-        <v>286</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="4" t="s">
+      <c r="B4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="I3" s="3">
-        <v>14</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="C4" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="I4" s="3">
-        <v>5</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>76</v>
+        <v>18</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" s="5">
+        <v>2</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="I5" s="3">
-        <v>56</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>76</v>
+        <v>24</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" s="11">
+        <v>80</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>60</v>
+        <v>15</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>20</v>
       </c>
       <c r="I6" s="3">
-        <v>6</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>76</v>
+        <v>285</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="12" t="s">
         <v>61</v>
       </c>
       <c r="I7" s="3">
-        <v>50</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>76</v>
+        <v>5</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D8" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="12" t="s">
         <v>62</v>
       </c>
       <c r="I8" s="3">
-        <v>115</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>76</v>
+        <v>5</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D9" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="12" t="s">
         <v>63</v>
       </c>
       <c r="I9" s="3">
-        <v>496</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>76</v>
+        <v>57</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D10" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="12" t="s">
         <v>64</v>
       </c>
       <c r="I10" s="3">
-        <v>10</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>76</v>
+        <v>6</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D11" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="12" t="s">
         <v>65</v>
       </c>
       <c r="I11" s="3">
-        <v>6</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>76</v>
+        <v>50</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D12" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="12" t="s">
         <v>66</v>
       </c>
       <c r="I12" s="3">
-        <v>3</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>76</v>
+        <v>115</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D13" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="12" t="s">
         <v>67</v>
       </c>
       <c r="I13" s="3">
-        <v>76</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>76</v>
+        <v>473</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D14" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="12" t="s">
         <v>68</v>
       </c>
       <c r="I14" s="3">
-        <v>71</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>76</v>
+        <v>10</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D15" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="12" t="s">
         <v>69</v>
       </c>
       <c r="I15" s="3">
-        <v>8</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>76</v>
+        <v>6</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>70</v>
+        <v>16</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="I16" s="3">
-        <v>4</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>76</v>
+        <v>2</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>71</v>
+        <v>46</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>70</v>
       </c>
       <c r="I17" s="3">
-        <v>5</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>72</v>
+        <v>17</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>22</v>
       </c>
       <c r="I18" s="3">
-        <v>26</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>73</v>
+      <c r="C19" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>71</v>
       </c>
       <c r="I19" s="3">
-        <v>7</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>76</v>
+        <v>8</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>74</v>
+      <c r="C20" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>72</v>
       </c>
       <c r="I20" s="3">
-        <v>287</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>76</v>
+        <v>4</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="C21" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="I21" s="3">
+        <v>5</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="B22" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="C22" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="I22" s="3">
+        <v>26</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="I21" s="3">
-        <v>257</v>
-      </c>
-      <c r="J21" s="2" t="s">
+      <c r="I23" s="3">
+        <v>7</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D24" s="12" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="I22" s="8">
-        <v>2</v>
-      </c>
-      <c r="J22" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="I23" s="8">
-        <v>4</v>
-      </c>
-      <c r="J23" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="I24" s="8">
-        <v>2</v>
-      </c>
-      <c r="J24" s="2" t="s">
-        <v>77</v>
+      <c r="I24" s="3">
+        <v>280</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>20</v>
+        <v>59</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D25" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="I25" s="12">
-        <v>80</v>
-      </c>
-      <c r="J25" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="I25" s="3">
+        <v>257</v>
+      </c>
+      <c r="J25" s="1" t="s">
         <v>78</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="A5">
+    <cfRule type="duplicateValues" dxfId="10" priority="2700"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A1:B1">
-    <cfRule type="duplicateValues" dxfId="15" priority="140"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="2480"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:H1">
-    <cfRule type="duplicateValues" dxfId="6" priority="141"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="142" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="2691"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="2692" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1">
-    <cfRule type="duplicateValues" dxfId="4" priority="138"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="139" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="2478"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="2479" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:L1">
-    <cfRule type="duplicateValues" dxfId="2" priority="136"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="137" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="2476"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="2477" stopIfTrue="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A25">
-    <cfRule type="duplicateValues" dxfId="0" priority="144"/>
+  <conditionalFormatting sqref="A16:A17">
+    <cfRule type="duplicateValues" dxfId="2" priority="2704"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2705"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A6:A25">
+    <cfRule type="duplicateValues" dxfId="0" priority="2712"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>